<commit_message>
auditor: RGF quadrimestral nos quadros 6 e 7
O RGF passou a ser publicado por quadrimestre. A tela de auditoria troca os
campos RGF 1º/2º Semestre por RGF 1º/2º/3º Quadrimestre.

- Q7: le a Tabela 2.0 do RGF do 3º quadrimestre (Anterior + 1º/2º/3º quad).
  O extrator antigo procurava a Tabela 2.3 e pegava so 3 das 4 colunas,
  jogando o 2º quadrimestre na coluna de fim de ano. Template e RIT passam
  a ter 3 colunas de quadrimestre.
- Q6: a coluna "1º Semestre" vira "2º Quadrimestre" (RGF do 2º quad);
  "Apurado pelo TCE" vem do RGF do 3º quad.
- RGF semestral continua aceito pela API (rgf1semestre/rgf2semestre) como
  fallback.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend-auditor/templates/quadro_06.xlsx
+++ b/backend-auditor/templates/quadro_06.xlsx
@@ -1,140 +1,65 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\claud\Desktop\auditor_tce6\kora\templates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB2010A6-9CC4-4121-8146-16EE6A890443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Planilha1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
-  <si>
-    <t>Quadro 6 – Comportamento da Despesa com Pessoal no Exercício</t>
-  </si>
-  <si>
-    <t>1º Semestre(R$)</t>
-  </si>
-  <si>
-    <t>(APURADO PELO TCE) (R$)</t>
-  </si>
-  <si>
-    <t>Total Despesa</t>
-  </si>
-  <si>
-    <t>RECEITA CORRENTE LÍQUIDA</t>
-  </si>
-  <si>
-    <t>RECEITA CORRENTE LÍQUIDA )</t>
-  </si>
-  <si>
-    <t>Despesa de Pessoal EXECUTIVO – Limite Legal - 54% do RCL - art. 21 II da LRF</t>
-  </si>
-  <si>
-    <t>Percentual e Valor Apurados</t>
-  </si>
-  <si>
-    <t>Este quadro demonstra o comportamento da despesa de pessoal no exercício corrente do Município.</t>
-  </si>
-  <si>
-    <t>{quadro_6_despesa_pessoal.primeiro_semestre.total_despesa}</t>
-  </si>
-  <si>
-    <t>{quadro_6_despesa_pessoal.primeiro_semestre.receita_corrente_liquida}</t>
-  </si>
-  <si>
-    <t>{quadro_6_despesa_pessoal.primeiro_semestre.limite_legal_54_pct}</t>
-  </si>
-  <si>
-    <t>{quadro_6_despesa_pessoal.primeiro_semestre.percentual_apurado}</t>
-  </si>
-  <si>
-    <t>{quadro_6_despesa_pessoal.apurado_pelo_tce.total_despesa}</t>
-  </si>
-  <si>
-    <t>{quadro_6_despesa_pessoal.apurado_pelo_tce.receita_corrente_liquida}</t>
-  </si>
-  <si>
-    <t>{quadro_6_despesa_pessoal.apurado_pelo_tce.limite_legal_54_pct}</t>
-  </si>
-  <si>
-    <t>{quadro_6_despesa_pessoal.apurado_pelo_tce.percentual_apurado}</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$R$-416]\ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF7A5C00"/>
       <sz val="13"/>
-      <color rgb="FF7A5C00"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <i/>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF595959"/>
       <sz val="10"/>
-      <color rgb="FF595959"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="6">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -192,53 +117,112 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="13">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -557,145 +541,167 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="438" row="2">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{60E7AD35-7BD7-4302-9D8F-B6D5AD800741}">
-  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="claude.fileId" value="&quot;d07dc8f8-9d4f-4dc7-b1e5-6a1c186cc1e6&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D35"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="42.5546875" customWidth="1"/>
-    <col min="2" max="2" width="22.21875" customWidth="1"/>
-    <col min="3" max="3" width="42.5546875" customWidth="1"/>
-    <col min="4" max="4" width="33.77734375" customWidth="1"/>
-    <col min="5" max="5" width="24.109375" customWidth="1"/>
+    <col width="42.5546875" customWidth="1" min="1" max="1"/>
+    <col width="22.21875" customWidth="1" min="2" max="2"/>
+    <col width="42.5546875" customWidth="1" min="3" max="3"/>
+    <col width="33.77734375" customWidth="1" min="4" max="4"/>
+    <col width="24.109375" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="25.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
+    <row r="1" ht="25.95" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Quadro 6 – Comportamento da Despesa com Pessoal no Exercício</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>8</v>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Este quadro demonstra o comportamento da despesa de pessoal no exercício corrente do Município.</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:4" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="4"/>
+    <row r="3" ht="15" customHeight="1"/>
+    <row r="4" ht="34.05" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2º Quadrimestre (R$)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>(APURADO PELO TCE) (R$)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n"/>
     </row>
-    <row r="5" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>13</v>
+    <row r="5" ht="22.05" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Total Despesa</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>{quadro_6_despesa_pessoal.segundo_quadrimestre.total_despesa}</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Total Despesa</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>{quadro_6_despesa_pessoal.apurado_pelo_tce.total_despesa}</t>
+        </is>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>14</v>
+    <row r="6" ht="22.05" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>RECEITA CORRENTE LÍQUIDA</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>{quadro_6_despesa_pessoal.segundo_quadrimestre.receita_corrente_liquida}</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>RECEITA CORRENTE LÍQUIDA )</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>{quadro_6_despesa_pessoal.apurado_pelo_tce.receita_corrente_liquida}</t>
+        </is>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>15</v>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Despesa de Pessoal EXECUTIVO – Limite Legal - 54% do RCL - art. 21 II da LRF</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>{quadro_6_despesa_pessoal.segundo_quadrimestre.limite_legal_54_pct}</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Despesa de Pessoal EXECUTIVO – Limite Legal - 54% do RCL - art. 21 II da LRF</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>{quadro_6_despesa_pessoal.apurado_pelo_tce.limite_legal_54_pct}</t>
+        </is>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>16</v>
+    <row r="8" ht="22.05" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Percentual e Valor Apurados</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>{quadro_6_despesa_pessoal.segundo_quadrimestre.percentual_apurado}</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Percentual e Valor Apurados</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>{quadro_6_despesa_pessoal.apurado_pelo_tce.percentual_apurado}</t>
+        </is>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="19" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="20" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="21" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="24" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="25" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="26" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="27" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="28" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="29" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="30" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="31" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="32" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="33" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="34" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="35" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="9" ht="22.05" customHeight="1"/>
+    <row r="10" ht="22.05" customHeight="1"/>
+    <row r="11" ht="22.05" customHeight="1"/>
+    <row r="12" ht="22.05" customHeight="1"/>
+    <row r="13" ht="22.05" customHeight="1"/>
+    <row r="14" ht="22.05" customHeight="1"/>
+    <row r="15" ht="22.05" customHeight="1"/>
+    <row r="16" ht="19.95" customHeight="1"/>
+    <row r="17" ht="19.95" customHeight="1"/>
+    <row r="18" ht="19.95" customHeight="1"/>
+    <row r="19" ht="19.95" customHeight="1"/>
+    <row r="20" ht="19.95" customHeight="1"/>
+    <row r="21" ht="19.95" customHeight="1"/>
+    <row r="22" ht="19.95" customHeight="1"/>
+    <row r="23" ht="19.95" customHeight="1"/>
+    <row r="24" ht="19.95" customHeight="1"/>
+    <row r="25" ht="19.95" customHeight="1"/>
+    <row r="26" ht="19.95" customHeight="1"/>
+    <row r="27" ht="19.95" customHeight="1"/>
+    <row r="28" ht="19.95" customHeight="1"/>
+    <row r="29" ht="19.95" customHeight="1"/>
+    <row r="30" ht="19.95" customHeight="1"/>
+    <row r="31" ht="19.95" customHeight="1"/>
+    <row r="32" ht="19.95" customHeight="1"/>
+    <row r="33" ht="19.95" customHeight="1"/>
+    <row r="34" ht="19.95" customHeight="1"/>
+    <row r="35" ht="19.95" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
 </worksheet>
 </file>
</xml_diff>